<commit_message>
update target release dates
</commit_message>
<xml_diff>
--- a/tools/latest.xlsx
+++ b/tools/latest.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10911"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucifer/vscode_Luci_scripts/HBCD-DOCS/hbcd-docs-internal/tools/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15CE57FA-1280-9A42-AC04-C5EE3F24F43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="🤩 public data release" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="🤩 public data release"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -289,6 +283,9 @@
     <t>C-PACEs</t>
   </si>
   <si>
+    <t>Summary scores for `sed_bm_paces` are currently calculated as the sum of individual item responses rather than the average. Until corrected, users may compute their own average-based summary scores using the item-level data provided in the dataset.</t>
+  </si>
+  <si>
     <t>[DATA ERROR] - 2 corrupt files in MRI raw BIDS (func)</t>
   </si>
   <si>
@@ -433,6 +430,9 @@
     <t>On hold- need more info</t>
   </si>
   <si>
+    <t>Instruction</t>
+  </si>
+  <si>
     <t>Instruction text in each form&amp;apos;s metadata is automatically extracted from the most recent `instruction` field in the REDCap Data Dictionary (based on field order). Because this process is automated, it may produce the following issues: (1) If an instruction spans multiple fields, only the last portion will be captured and/or (2) Some fields may display text intended for a previous section. Until this is corrected, please refer to original forms for accurate instruction text.</t>
   </si>
   <si>
@@ -451,6 +451,9 @@
     <t>MLDS</t>
   </si>
   <si>
+    <t>Total non-parental hours/week (`ncl_ch_mlds_arr_hr_wk`) includes implausible values due to data entry errors. Exclude values &gt;168 hours from analysis.</t>
+  </si>
+  <si>
     <t>[FUTURE DATA CORRECTION]- "does not apply" should = 8 for ECBQ</t>
   </si>
   <si>
@@ -550,6 +553,9 @@
     <t>EPDS</t>
   </si>
   <si>
+    <t xml:space="preserve"> Some V01-V03 records show inconsistencies between item responses and the calculated sum score, including (1) items present, but sum score is null; (2) items null, but sum score is 0.</t>
+  </si>
+  <si>
     <t>Anthro: ph_ch_anthro_head_for_age_boys_z_score</t>
   </si>
   <si>
@@ -562,6 +568,9 @@
     <t>APA 1/2</t>
   </si>
   <si>
+    <t>APA Level 2 was sometimes administered despite unmet gating criteria (e.g., missing Level 1 responses). These cases are not scored (“No additional inquiry required”) even when Level 2 responses are present. Level 2 item data will be removed to avoid confusion.</t>
+  </si>
+  <si>
     <t>[DD+DATA ERROR] Nail type field added for 2.0 all "Unknown"</t>
   </si>
   <si>
@@ -577,9 +586,15 @@
     <t>Healthv2 Preg</t>
   </si>
   <si>
+    <t>The field for the date when PNV was stopped (`pex_bm_healthv2_preg__exp__pnv_007__01`) is blank, despite participants having reported stopping.</t>
+  </si>
+  <si>
     <t>[LORIS TO REVIEW]- aspirin items in health v2 preg</t>
   </si>
   <si>
+    <t>Note that items about aspirin use (`pex_bm_healthv2_preg__exp__pnv_{011|012}`) are largely blank.</t>
+  </si>
+  <si>
     <t>[DATA REQUEST]- consistent ICD code names</t>
   </si>
   <si>
@@ -604,9 +619,15 @@
     <t>Data Type</t>
   </si>
   <si>
+    <t>Summary score variables in the Bayley and CDI are misclassified as text in the metadata, which may cause formatting issues in some tools.</t>
+  </si>
+  <si>
     <t>DD &amp;apos;instruction&amp;apos; field all blank</t>
   </si>
   <si>
+    <t>The &amp;apos;instruction&amp;apos; Data Dictionary element is currently blank.</t>
+  </si>
+  <si>
     <t>EEG file was not re-id&amp;apos;d (put in RTD) need to dig into how it happened -</t>
   </si>
   <si>
@@ -683,40 +704,14 @@
   </si>
   <si>
     <t>Tabulated XCP-D Myers-Labonte tables (`img_xcpd_hash-{X}_space-fsLR_seg-MyersLabonte_stat-mean_desc-_morph`) metadata will be corrected to have a `sub_domain` value of `Structural MRI` (currently `Resting State fMRI`).</t>
-  </si>
-  <si>
-    <t>Instruction</t>
-  </si>
-  <si>
-    <t>Summary score variables in the Bayley and CDI are misclassified as text in the metadata, which may cause formatting issues in some tools.</t>
-  </si>
-  <si>
-    <t>Total non-parental hours/week (`ncl_ch_mlds_arr_hr_wk`) includes implausible values due to data entry errors. Exclude values &gt;168 hours from analysis.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Some V01-V03 records show inconsistencies between item responses and the calculated sum score, including (1) items present, but sum score is null; (2) items null, but sum score is 0.</t>
-  </si>
-  <si>
-    <t>The field for the date when PNV was stopped (`pex_bm_healthv2_preg__exp__pnv_007__01`) is blank, despite participants having reported stopping.</t>
-  </si>
-  <si>
-    <t>Note that items about aspirin use (`pex_bm_healthv2_preg__exp__pnv_{011|012}`) are largely blank.</t>
-  </si>
-  <si>
-    <t>Summary scores for `sed_bm_paces` are currently calculated as the sum of individual item responses rather than the average. Until corrected, users may compute their own average-based summary scores using the item-level data provided in the dataset.</t>
-  </si>
-  <si>
-    <t>APA Level 2 was sometimes administered despite unmet gating criteria (e.g., missing Level 1 responses). These cases are not scored (“No additional inquiry required”) even when Level 2 responses are present. Level 2 item data will be removed to avoid confusion.</t>
-  </si>
-  <si>
-    <t>The &amp;apos;instruction&amp;apos; Data Dictionary element is currently blank.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -739,13 +734,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFffffff"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -759,42 +748,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD6D6D6"/>
+        <fgColor rgb="FFd6d6d6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC4C4C4"/>
+        <fgColor rgb="FFc4c4c4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF007F"/>
+        <fgColor rgb="FFff007f"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9D99B9"/>
+        <fgColor rgb="FF9d99b9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00C875"/>
+        <fgColor rgb="FF00c875"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF66CCFF"/>
+        <fgColor rgb="FF66ccff"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF007EB5"/>
+        <fgColor rgb="FF007eb5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFDAB3D"/>
+        <fgColor rgb="FFfdab3d"/>
       </patternFill>
     </fill>
     <fill>
@@ -804,47 +793,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDF2F4A"/>
+        <fgColor rgb="FFdf2f4a"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9D50DD"/>
+        <fgColor rgb="FF9d50dd"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF6D3B"/>
+        <fgColor rgb="FFff6d3b"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBB3354"/>
+        <fgColor rgb="FFbb3354"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCAB641"/>
+        <fgColor rgb="FFcab641"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9CD326"/>
+        <fgColor rgb="FF9cd326"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCB00"/>
+        <fgColor rgb="FFffcb00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF563E3E"/>
+        <fgColor rgb="FF563e3e"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF5AC4"/>
+        <fgColor rgb="FFff5ac4"/>
       </patternFill>
     </fill>
   </fills>
@@ -858,16 +847,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </left>
       <right style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </right>
       <top style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -882,101 +871,107 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="31">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="15" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="16" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="17" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="18" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="19" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -987,10 +982,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1028,71 +1023,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1120,7 +1115,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1143,11 +1138,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1156,13 +1151,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1172,7 +1167,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1181,7 +1176,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1190,7 +1185,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1198,10 +1193,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1266,22 +1261,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:L70"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" style="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20" style="28" bestFit="1" customWidth="1"/>
-    <col min="4" max="10" width="20" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="255.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="28" width="40.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="29" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="30" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="28" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="28" width="255.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="28" width="20.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1319,7 +1320,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
@@ -1351,7 +1352,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
@@ -1379,7 +1380,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
@@ -1411,7 +1412,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="4" t="s">
         <v>31</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="4" t="s">
         <v>36</v>
       </c>
@@ -1475,12 +1476,16 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="6"/>
+      <c r="B7" s="5">
+        <v>2.1</v>
+      </c>
+      <c r="C7" s="6">
+        <v>21.1</v>
+      </c>
       <c r="D7" s="7"/>
       <c r="E7" s="8" t="s">
         <v>37</v>
@@ -1507,7 +1512,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4" t="s">
         <v>46</v>
       </c>
@@ -1539,7 +1544,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1571,7 +1576,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="4" t="s">
         <v>52</v>
       </c>
@@ -1603,7 +1608,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="4" t="s">
         <v>54</v>
       </c>
@@ -1639,7 +1644,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="4" t="s">
         <v>56</v>
       </c>
@@ -1675,7 +1680,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="4" t="s">
         <v>59</v>
       </c>
@@ -1711,7 +1716,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="4" t="s">
         <v>62</v>
       </c>
@@ -1747,7 +1752,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="4" t="s">
         <v>66</v>
       </c>
@@ -1783,7 +1788,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="20">
       <c r="A16" s="4" t="s">
         <v>71</v>
       </c>
@@ -1819,7 +1824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="20">
       <c r="A17" s="4" t="s">
         <v>76</v>
       </c>
@@ -1853,7 +1858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="20">
       <c r="A18" s="4" t="s">
         <v>80</v>
       </c>
@@ -1887,7 +1892,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="20">
       <c r="A19" s="4" t="s">
         <v>83</v>
       </c>
@@ -1921,7 +1926,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="20">
       <c r="A20" s="4" t="s">
         <v>87</v>
       </c>
@@ -1951,22 +1956,22 @@
         <v>88</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>227</v>
+        <v>89</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="20">
       <c r="A21" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21" s="20">
         <v>2.1</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>16</v>
@@ -1981,21 +1986,21 @@
         <v>33</v>
       </c>
       <c r="I21" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="20">
       <c r="A22" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B22" s="20">
         <v>2.1</v>
@@ -2008,10 +2013,10 @@
         <v>67</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>15</v>
@@ -2020,18 +2025,18 @@
         <v>16</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L22" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="20">
       <c r="A23" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B23" s="20">
         <v>2.1</v>
@@ -2056,18 +2061,18 @@
         <v>16</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L23" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="20">
       <c r="A24" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B24" s="20">
         <v>2.1</v>
@@ -2090,18 +2095,18 @@
         <v>16</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L24" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="20">
       <c r="A25" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B25" s="20">
         <v>2.1</v>
@@ -2129,15 +2134,15 @@
         <v>40</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L25" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="20">
       <c r="A26" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B26" s="20">
         <v>2.1</v>
@@ -2165,15 +2170,15 @@
         <v>40</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L26" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="20">
       <c r="A27" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B27" s="20">
         <v>2.1</v>
@@ -2198,18 +2203,18 @@
         <v>16</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L27" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="20">
       <c r="A28" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="20">
@@ -2232,18 +2237,18 @@
         <v>16</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K28" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="L28" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="20">
       <c r="A29" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="20">
@@ -2266,18 +2271,18 @@
         <v>16</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K29" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="L29" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="20">
       <c r="A30" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B30" s="22">
         <v>3</v>
@@ -2300,18 +2305,18 @@
         <v>16</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K30" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="L30" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="20">
       <c r="A31" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="6"/>
@@ -2332,18 +2337,18 @@
         <v>16</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K31" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L31" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="20">
       <c r="A32" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B32" s="22">
         <v>3</v>
@@ -2366,18 +2371,18 @@
         <v>16</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K32" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="L32" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="20">
       <c r="A33" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B33" s="22">
         <v>3</v>
@@ -2400,18 +2405,18 @@
         <v>16</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K33" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="L33" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="20">
       <c r="A34" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B34" s="22">
         <v>3</v>
@@ -2434,18 +2439,18 @@
         <v>16</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K34" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L34" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="20">
       <c r="A35" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="6"/>
@@ -2466,18 +2471,18 @@
         <v>16</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K35" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L35" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="20">
       <c r="A36" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B36" s="22">
         <v>3</v>
@@ -2497,21 +2502,21 @@
         <v>33</v>
       </c>
       <c r="I36" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>221</v>
+        <v>138</v>
       </c>
       <c r="K36" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L36" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="20">
       <c r="A37" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B37" s="22">
         <v>3</v>
@@ -2534,18 +2539,18 @@
         <v>16</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K37" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L37" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="20">
       <c r="A38" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B38" s="22">
         <v>3</v>
@@ -2568,18 +2573,18 @@
         <v>16</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="K38" s="29" t="s">
-        <v>223</v>
+        <v>144</v>
+      </c>
+      <c r="K38" s="27" t="s">
+        <v>145</v>
       </c>
       <c r="L38" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="20">
       <c r="A39" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B39" s="22">
         <v>3</v>
@@ -2602,18 +2607,18 @@
         <v>16</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="K39" s="11" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="L39" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="20">
       <c r="A40" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B40" s="22">
         <v>3</v>
@@ -2636,18 +2641,18 @@
         <v>16</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="K40" s="11" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="L40" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="20">
       <c r="A41" s="4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B41" s="22">
         <v>3</v>
@@ -2673,15 +2678,15 @@
         <v>50</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="L41" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="20">
       <c r="A42" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B42" s="22">
         <v>3</v>
@@ -2704,18 +2709,18 @@
         <v>16</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="K42" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="L42" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="20">
       <c r="A43" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B43" s="22">
         <v>3</v>
@@ -2738,18 +2743,18 @@
         <v>16</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="K43" s="11" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="L43" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="20">
       <c r="A44" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B44" s="22">
         <v>3</v>
@@ -2775,15 +2780,15 @@
         <v>50</v>
       </c>
       <c r="K44" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="L44" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="20">
       <c r="A45" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="6"/>
@@ -2792,7 +2797,7 @@
         <v>13</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>14</v>
@@ -2804,18 +2809,18 @@
         <v>16</v>
       </c>
       <c r="J45" s="11" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="K45" s="11" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="L45" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="20">
       <c r="A46" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B46" s="22">
         <v>3</v>
@@ -2823,7 +2828,7 @@
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
       <c r="E46" s="17" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F46" s="24" t="s">
         <v>68</v>
@@ -2832,22 +2837,22 @@
         <v>68</v>
       </c>
       <c r="H46" s="17" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>16</v>
       </c>
       <c r="J46" s="11" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="K46" s="11"/>
       <c r="L46" s="16" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="20">
       <c r="A47" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B47" s="22">
         <v>3</v>
@@ -2870,18 +2875,18 @@
         <v>16</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="K47" s="11" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="L47" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="20">
       <c r="A48" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B48" s="22">
         <v>3</v>
@@ -2904,18 +2909,18 @@
         <v>16</v>
       </c>
       <c r="J48" s="11" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="K48" s="11" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="L48" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="20">
       <c r="A49" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B49" s="22">
         <v>3</v>
@@ -2938,18 +2943,18 @@
         <v>16</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="K49" t="s">
-        <v>224</v>
+        <v>178</v>
+      </c>
+      <c r="K49" s="27" t="s">
+        <v>179</v>
       </c>
       <c r="L49" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="50" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="20">
       <c r="A50" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B50" s="22">
         <v>3</v>
@@ -2975,15 +2980,15 @@
         <v>50</v>
       </c>
       <c r="K50" s="11" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="L50" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="20">
       <c r="A51" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B51" s="22">
         <v>3</v>
@@ -3006,24 +3011,24 @@
         <v>16</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="K51" s="11" t="s">
-        <v>228</v>
+        <v>184</v>
       </c>
       <c r="L51" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="20">
       <c r="A52" s="4" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B52" s="5"/>
       <c r="C52" s="6"/>
       <c r="D52" s="7"/>
       <c r="E52" s="25" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="F52" s="24" t="s">
         <v>68</v>
@@ -3041,15 +3046,15 @@
         <v>81</v>
       </c>
       <c r="K52" s="11" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="L52" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="20">
       <c r="A53" s="4" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B53" s="5"/>
       <c r="C53" s="6"/>
@@ -3070,18 +3075,18 @@
         <v>16</v>
       </c>
       <c r="J53" s="11" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="K53" s="11" t="s">
-        <v>225</v>
+        <v>190</v>
       </c>
       <c r="L53" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="20">
       <c r="A54" s="4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="6"/>
@@ -3102,18 +3107,18 @@
         <v>16</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="K54" s="11" t="s">
-        <v>226</v>
+        <v>192</v>
       </c>
       <c r="L54" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="55" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="20">
       <c r="A55" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B55" s="22">
         <v>3</v>
@@ -3136,18 +3141,18 @@
         <v>16</v>
       </c>
       <c r="J55" s="11" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="K55" s="11" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="L55" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="20">
       <c r="A56" s="4" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B56" s="22">
         <v>3</v>
@@ -3177,9 +3182,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="20">
       <c r="A57" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B57" s="22">
         <v>3</v>
@@ -3207,9 +3212,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="20">
       <c r="A58" s="4" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B58" s="22">
         <v>3</v>
@@ -3217,7 +3222,7 @@
       <c r="C58" s="6"/>
       <c r="D58" s="7"/>
       <c r="E58" s="15" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="F58" s="25" t="s">
         <v>77</v>
@@ -3232,18 +3237,18 @@
         <v>16</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>193</v>
-      </c>
-      <c r="K58" t="s">
-        <v>222</v>
+        <v>200</v>
+      </c>
+      <c r="K58" s="27" t="s">
+        <v>201</v>
       </c>
       <c r="L58" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="59" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="20">
       <c r="A59" s="4" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B59" s="22">
         <v>3</v>
@@ -3266,18 +3271,18 @@
         <v>16</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>221</v>
+        <v>138</v>
       </c>
       <c r="K59" s="11" t="s">
-        <v>229</v>
+        <v>203</v>
       </c>
       <c r="L59" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="60" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="20">
       <c r="A60" s="4" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="B60" s="20">
         <v>2.1</v>
@@ -3286,7 +3291,7 @@
         <v>21.1</v>
       </c>
       <c r="D60" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E60" s="10" t="s">
         <v>16</v>
@@ -3301,21 +3306,21 @@
         <v>33</v>
       </c>
       <c r="I60" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="K60" s="11" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="L60" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="20">
       <c r="A61" s="4" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B61" s="20">
         <v>2.1</v>
@@ -3324,7 +3329,7 @@
         <v>21</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>16</v>
@@ -3339,21 +3344,21 @@
         <v>15</v>
       </c>
       <c r="I61" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="K61" s="11" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="L61" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="20">
       <c r="A62" s="4" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="B62" s="20">
         <v>2.1</v>
@@ -3362,7 +3367,7 @@
         <v>21</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>16</v>
@@ -3377,21 +3382,21 @@
         <v>33</v>
       </c>
       <c r="I62" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J62" s="11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K62" s="11" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="L62" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="20">
       <c r="A63" s="4" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="B63" s="20">
         <v>2.1</v>
@@ -3400,7 +3405,7 @@
         <v>21</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>16</v>
@@ -3415,21 +3420,21 @@
         <v>33</v>
       </c>
       <c r="I63" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J63" s="11" t="s">
         <v>40</v>
       </c>
       <c r="K63" s="11" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="L63" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="20">
       <c r="A64" s="4" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="B64" s="20">
         <v>2.1</v>
@@ -3438,7 +3443,7 @@
         <v>21</v>
       </c>
       <c r="D64" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>16</v>
@@ -3453,21 +3458,21 @@
         <v>33</v>
       </c>
       <c r="I64" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="K64" s="11" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="L64" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="20">
       <c r="A65" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="B65" s="20">
         <v>2.1</v>
@@ -3476,7 +3481,7 @@
         <v>21</v>
       </c>
       <c r="D65" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>16</v>
@@ -3491,21 +3496,21 @@
         <v>15</v>
       </c>
       <c r="I65" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J65" s="11" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="K65" s="11" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="L65" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="20">
       <c r="A66" s="4" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="B66" s="20">
         <v>2.1</v>
@@ -3514,7 +3519,7 @@
         <v>21</v>
       </c>
       <c r="D66" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E66" s="10" t="s">
         <v>16</v>
@@ -3529,21 +3534,21 @@
         <v>15</v>
       </c>
       <c r="I66" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J66" s="11" t="s">
         <v>44</v>
       </c>
       <c r="K66" s="11" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="L66" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="20">
       <c r="A67" s="4" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="B67" s="20">
         <v>2.1</v>
@@ -3552,7 +3557,7 @@
         <v>21</v>
       </c>
       <c r="D67" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>16</v>
@@ -3567,21 +3572,21 @@
         <v>15</v>
       </c>
       <c r="I67" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="K67" s="11" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="L67" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="20">
       <c r="A68" s="4" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="B68" s="20">
         <v>2.1</v>
@@ -3590,7 +3595,7 @@
         <v>21</v>
       </c>
       <c r="D68" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E68" s="10" t="s">
         <v>16</v>
@@ -3605,21 +3610,21 @@
         <v>33</v>
       </c>
       <c r="I68" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="K68" s="11" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="L68" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="69" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="20">
       <c r="A69" s="4" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B69" s="20">
         <v>2.1</v>
@@ -3628,7 +3633,7 @@
         <v>21</v>
       </c>
       <c r="D69" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>16</v>
@@ -3643,21 +3648,31 @@
         <v>33</v>
       </c>
       <c r="I69" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="K69" s="11" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="L69" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="20">
+      <c r="A70" s="27"/>
       <c r="B70" s="5"/>
       <c r="C70" s="6"/>
+      <c r="D70" s="27"/>
+      <c r="E70" s="27"/>
+      <c r="F70" s="27"/>
+      <c r="G70" s="27"/>
+      <c r="H70" s="27"/>
+      <c r="I70" s="27"/>
+      <c r="J70" s="27"/>
+      <c r="K70" s="27"/>
+      <c r="L70" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update KI and add BR 21.2 page
</commit_message>
<xml_diff>
--- a/tools/latest.xlsx
+++ b/tools/latest.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10911"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D458A66-823B-8946-89F5-2B25D1C11D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2E07A9-077B-7643-A314-915E817C6592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="🤩 public data release" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="249">
   <si>
     <t>Name</t>
   </si>
@@ -128,27 +128,27 @@
     <t>Anthro: LT goal for implementing score calculation in ETL based on EDD</t>
   </si>
   <si>
+    <t>21.1</t>
+  </si>
+  <si>
+    <t>Physical Health</t>
+  </si>
+  <si>
+    <t>Archived to BR</t>
+  </si>
+  <si>
+    <t>Growth</t>
+  </si>
+  <si>
+    <t>Add age-based z-scores to `ph_ch_anthro` (see [Z-Scores Excluded](https://docs.hbcdstudy.org/latest/instruments/physhealth/growth/#warning)).</t>
+  </si>
+  <si>
+    <t>Genomics - OLINK data proteomics</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Waiting on WG feedback</t>
-  </si>
-  <si>
-    <t>Physical Health</t>
-  </si>
-  <si>
-    <t>Archived to BR</t>
-  </si>
-  <si>
-    <t>Growth</t>
-  </si>
-  <si>
-    <t>Add age-based z-scores to `ph_ch_anthro` (see [Z-Scores Excluded](https://docs.hbcdstudy.org/latest/instruments/physhealth/growth/#warning)).</t>
-  </si>
-  <si>
-    <t>Genomics - OLINK data proteomics</t>
-  </si>
-  <si>
     <t>Active</t>
   </si>
   <si>
@@ -161,21 +161,6 @@
     <t>Add Olink Explore 384 Inflammation 1 Panel, proteomics measure of maternal inflammation during pregnancy</t>
   </si>
   <si>
-    <t>Bayley item-level scores</t>
-  </si>
-  <si>
-    <t>21.1</t>
-  </si>
-  <si>
-    <t>Neurocognition &amp; Language</t>
-  </si>
-  <si>
-    <t>Bayley-4</t>
-  </si>
-  <si>
-    <t>Add item-level scores.</t>
-  </si>
-  <si>
     <t>[DATA ERROR]- Study Navigator blank checkboxes</t>
   </si>
   <si>
@@ -234,9 +219,6 @@
   </si>
   <si>
     <t>[DATA ERROR]- PA/greenspace type_Data= text so breaking lasso dashboard</t>
-  </si>
-  <si>
-    <t>LORIS reviewing</t>
   </si>
   <si>
     <t>ecPROMIS-PAGS</t>
@@ -321,7 +303,7 @@
     <t>Not started yet</t>
   </si>
   <si>
-    <t>The Data Dictionary element `type_data` for `average_bmi` will be corrected to `double` (currently=`character`).</t>
+    <t>The data dictionary element `type_data` for `average_bmi` will be corrected to `double` (currently=`character`).</t>
   </si>
   <si>
     <t>Add DICOMs to release</t>
@@ -369,90 +351,93 @@
     <t>Inclusion of Blood Spot Card Results data from USDTL.</t>
   </si>
   <si>
+    <t>DD 'instruction' field all blank</t>
+  </si>
+  <si>
+    <t>Instruction</t>
+  </si>
+  <si>
+    <t>The 'instruction' data dictionary element is currently blank.</t>
+  </si>
+  <si>
+    <t>Followup item: scanner info</t>
+  </si>
+  <si>
+    <t>Scanner Info</t>
+  </si>
+  <si>
+    <t>Scanner information must currently be parsed from raw BIDS data (specifically the scans .tsv files), as described [here](https://docs.hbcdstudy.org/latest/help/faq/#faq-scanner-info). Future releases will include a dedicated 'MRI Info' table that summarizes scanner information across participants, similar to the ABCD study ([see details](https://docs.abcdstudy.org/latest/documentation/imaging/admin.html#mr_y_adm__info)).</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST] ERICA - add age &amp; date_taken fields back to ERICA once corrected (post 2.1 patch)</t>
+  </si>
+  <si>
+    <t>Add all age and `date_taken` fields (currently excluded due to use of coding rather than visit dates).</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- ecPROMIS child-caregiver infant</t>
+  </si>
+  <si>
+    <t>ecPROMIS CC</t>
+  </si>
+  <si>
+    <t>N=12 V03 participants with &lt;3 item responses are incorrectly scored as `0` in `mh_cg_pms__cc__inf`; set values to null prior to analysis.</t>
+  </si>
+  <si>
+    <t>[IMAGING] Add Cook's distance to tabulated imaging data</t>
+  </si>
+  <si>
+    <t>Cook's Distance</t>
+  </si>
+  <si>
+    <t>Addition Cook's distance values computed for fMRI.</t>
+  </si>
+  <si>
+    <t>[2.0 SCORING CORRECTION NEEDED]- V03 MAPS-TL</t>
+  </si>
+  <si>
+    <t>MAPS-TL (&lt;1yr)</t>
+  </si>
+  <si>
+    <t>N=4 participants with no item responses are incorrectly scored as `0`; set values to null prior to analysis.</t>
+  </si>
+  <si>
+    <t>[SCORING CORRECTION NEEDED]- EPDS</t>
+  </si>
+  <si>
+    <t>LORIS reviewing</t>
+  </si>
+  <si>
+    <t>EPDS</t>
+  </si>
+  <si>
+    <t>Inconsistent scoring: (1) item responses present, but score is null (N=1); (2) all items null, but score is `0` (N≥3).</t>
+  </si>
+  <si>
+    <t>Anthro: ph_ch_anthro_head_for_age_boys_z_score</t>
+  </si>
+  <si>
+    <t>Growth (`ph_ch_anthro`) filter ranges will be updated to be visit-specific, as current ranges allow biologically implausible values (see [Range Checks](https://docs.hbcdstudy.org/latest/instruments/physhealth/growth/#warning)).</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST]-household roster - sex variable</t>
+  </si>
+  <si>
+    <t>Demo</t>
+  </si>
+  <si>
+    <t>Add household roster fields capturing the sex of listed individuals (adult &amp; child tables).</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST]- anthro z-score calcs when no EDD/adjusted age available</t>
+  </si>
+  <si>
+    <t>on hold/later</t>
+  </si>
+  <si>
     <t>TBD</t>
   </si>
   <si>
-    <t>DD 'instruction' field all blank</t>
-  </si>
-  <si>
-    <t>Instruction</t>
-  </si>
-  <si>
-    <t>The 'instruction' Data Dictionary element is currently blank.</t>
-  </si>
-  <si>
-    <t>Followup item: scanner info</t>
-  </si>
-  <si>
-    <t>Scanner Info</t>
-  </si>
-  <si>
-    <t>Scanner information must currently be parsed from raw BIDS data (specifically the scans .tsv files), as described [here](https://docs.hbcdstudy.org/latest/help/faq/#faq-scanner-info). Future releases will include a dedicated 'MRI Info' table that summarizes scanner information across participants, similar to the ABCD study ([see details](https://docs.abcdstudy.org/latest/documentation/imaging/admin.html#mr_y_adm__info)).</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST] ERICA - add age &amp; date_taken fields back to ERICA once corrected (post 2.1 patch)</t>
-  </si>
-  <si>
-    <t>Add all age and `date_taken` fields (currently excluded due to use of coding rather than visit dates).</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- ecPROMIS child-caregiver infant</t>
-  </si>
-  <si>
-    <t>ecPROMIS CC</t>
-  </si>
-  <si>
-    <t>N=12 V03 participants with &lt;3 item responses are incorrectly scored as `0` in `mh_cg_pms__cc__inf`; set values to null prior to analysis.</t>
-  </si>
-  <si>
-    <t>[IMAGING] Add Cook's distance to tabulated imaging data</t>
-  </si>
-  <si>
-    <t>Cook's Distance</t>
-  </si>
-  <si>
-    <t>Addition Cook's distance values computed for fMRI.</t>
-  </si>
-  <si>
-    <t>[2.0 SCORING CORRECTION NEEDED]- V03 MAPS-TL</t>
-  </si>
-  <si>
-    <t>MAPS-TL (&lt;1yr)</t>
-  </si>
-  <si>
-    <t>N=4 participants with no item responses are incorrectly scored as `0`; set values to null prior to analysis.</t>
-  </si>
-  <si>
-    <t>[SCORING CORRECTION NEEDED]- EPDS</t>
-  </si>
-  <si>
-    <t>EPDS</t>
-  </si>
-  <si>
-    <t>Inconsistent scoring: (1) item responses present, but score is null (N=1); (2) all items null, but score is `0` (N≥3).</t>
-  </si>
-  <si>
-    <t>Anthro: ph_ch_anthro_head_for_age_boys_z_score</t>
-  </si>
-  <si>
-    <t>Growth (`ph_ch_anthro`) filter ranges will be updated to be visit-specific, as current ranges allow biologically implausible values (see [Range Checks](https://docs.hbcdstudy.org/latest/instruments/physhealth/growth/#warning)).</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST]-household roster - sex variable</t>
-  </si>
-  <si>
-    <t>Demo</t>
-  </si>
-  <si>
-    <t>Add household roster fields capturing the sex of listed individuals (adult &amp; child tables).</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST]- anthro z-score calcs when no EDD/adjusted age available</t>
-  </si>
-  <si>
-    <t>on hold/later</t>
-  </si>
-  <si>
     <t>[DATA ERROR]- missing sleep score fields- ecPROMIS SLEEP</t>
   </si>
   <si>
@@ -501,6 +486,9 @@
     <t>EEG</t>
   </si>
   <si>
+    <t>Age fields</t>
+  </si>
+  <si>
     <t>Chronological and adjusted age fall outside of 3-9 months in N=74 V03 sessions (site entry errors); exclude age values prior to analysis.</t>
   </si>
   <si>
@@ -513,6 +501,30 @@
     <t>PNR data were incorrectly reported using TLFB versions 1/2 and will be updated to [version 3 specific to PNR](https://docs.hbcdstudy.org/latest/instruments/pregexp/su/tlfb/#v3).</t>
   </si>
   <si>
+    <t>Gabi raw BIDs</t>
+  </si>
+  <si>
+    <t>New; needs discussion</t>
+  </si>
+  <si>
+    <t>Novel Tech &amp; Wearable Sensors</t>
+  </si>
+  <si>
+    <t>GABI</t>
+  </si>
+  <si>
+    <t>Addition of raw BIDS data for GABI (infant heart rate).</t>
+  </si>
+  <si>
+    <t>[POSSIBLE DATA ERROR]- roster at V02 or V03</t>
+  </si>
+  <si>
+    <t>Started, outprioritized</t>
+  </si>
+  <si>
+    <t>Roster was inappropriately collected at V02/V03 for all cohorts and should have been restricted to V02 PNRs and alternate caregiver cohorts; to be excluded.</t>
+  </si>
+  <si>
     <t>Remove 'sequence' field from all tables in Lasso</t>
   </si>
   <si>
@@ -525,6 +537,9 @@
     <t>[DATA ERROR]-MLDS  total hours per week of non-parental hours</t>
   </si>
   <si>
+    <t>Neurocognition &amp; Language</t>
+  </si>
+  <si>
     <t>MLDS</t>
   </si>
   <si>
@@ -565,6 +580,9 @@
   </si>
   <si>
     <t>BISQR: infant sleep score - need to add</t>
+  </si>
+  <si>
+    <t>Waiting on WG feedback</t>
   </si>
   <si>
     <t>BISQ-SF</t>
@@ -770,7 +788,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -819,12 +837,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC4C4C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF563E3E"/>
+        <fgColor rgb="FFFAA1F1"/>
       </patternFill>
     </fill>
     <fill>
@@ -839,12 +852,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCB00"/>
+        <fgColor rgb="FFC4C4C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFAA1F1"/>
+        <fgColor rgb="FFFFCB00"/>
       </patternFill>
     </fill>
     <fill>
@@ -877,6 +890,21 @@
         <fgColor rgb="FFCAB641"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF037F4C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF563E3E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -890,7 +918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -956,6 +984,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1297,7 +1331,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1527,23 +1561,23 @@
       <c r="D7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>38</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>39</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>19</v>
@@ -1551,16 +1585,16 @@
     </row>
     <row r="8" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>44</v>
@@ -1571,8 +1605,8 @@
       <c r="G8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="14" t="s">
-        <v>40</v>
+      <c r="H8" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>46</v>
@@ -1592,22 +1626,22 @@
         <v>2.1</v>
       </c>
       <c r="C9" s="3">
-        <v>21.1</v>
-      </c>
-      <c r="D9" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="13" t="s">
         <v>50</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="14" t="s">
-        <v>40</v>
+      <c r="H9" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>51</v>
@@ -1627,28 +1661,28 @@
         <v>2.1</v>
       </c>
       <c r="C10" s="3">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>55</v>
+      <c r="E10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="14" t="s">
-        <v>40</v>
+      <c r="H10" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>19</v>
@@ -1656,7 +1690,7 @@
     </row>
     <row r="11" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B11" s="3">
         <v>2.1</v>
@@ -1667,23 +1701,23 @@
       <c r="D11" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>45</v>
+      <c r="E11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="14" t="s">
-        <v>40</v>
+      <c r="H11" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>19</v>
@@ -1691,7 +1725,7 @@
     </row>
     <row r="12" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B12" s="3">
         <v>2.1</v>
@@ -1699,26 +1733,26 @@
       <c r="C12" s="3">
         <v>21.1</v>
       </c>
-      <c r="D12" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>14</v>
+      <c r="D12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>60</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="14" t="s">
-        <v>40</v>
+      <c r="H12" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I12" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>19</v>
@@ -1726,13 +1760,13 @@
     </row>
     <row r="13" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B13" s="3">
         <v>2.1</v>
       </c>
       <c r="C13" s="3">
-        <v>21.1</v>
+        <v>21.2</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>12</v>
@@ -1741,19 +1775,19 @@
         <v>13</v>
       </c>
       <c r="F13" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G13" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="I13" s="3" t="s">
+      <c r="J13" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>67</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>19</v>
@@ -1761,7 +1795,7 @@
     </row>
     <row r="14" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" s="3">
         <v>2.1</v>
@@ -1772,23 +1806,23 @@
       <c r="D14" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="19" t="s">
+      <c r="E14" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>19</v>
@@ -1796,22 +1830,22 @@
     </row>
     <row r="15" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B15" s="3">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>39</v>
+        <v>43</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>38</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>15</v>
@@ -1820,10 +1854,10 @@
         <v>16</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>19</v>
@@ -1831,34 +1865,34 @@
     </row>
     <row r="16" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B16" s="3">
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>15</v>
+      <c r="F16" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>19</v>
@@ -1866,16 +1900,16 @@
     </row>
     <row r="17" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B17" s="3">
         <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>44</v>
@@ -1890,10 +1924,10 @@
         <v>16</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="K17" s="7" t="s">
         <v>19</v>
@@ -1901,34 +1935,34 @@
     </row>
     <row r="18" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>21</v>
+      <c r="F18" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>19</v>
@@ -1936,34 +1970,34 @@
     </row>
     <row r="19" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B19" s="3">
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F19" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>84</v>
+      <c r="F19" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>19</v>
@@ -1971,34 +2005,34 @@
     </row>
     <row r="20" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B20" s="3">
         <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F20" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>15</v>
+      <c r="F20" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H20" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>19</v>
@@ -2006,16 +2040,16 @@
     </row>
     <row r="21" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B21" s="3">
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>44</v>
@@ -2030,10 +2064,10 @@
         <v>16</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>19</v>
@@ -2041,16 +2075,16 @@
     </row>
     <row r="22" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B22" s="3">
         <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>44</v>
@@ -2058,17 +2092,17 @@
       <c r="F22" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G22" s="8" t="s">
-        <v>21</v>
+      <c r="G22" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H22" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K22" s="7" t="s">
         <v>19</v>
@@ -2076,34 +2110,34 @@
     </row>
     <row r="23" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B23" s="3">
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>97</v>
+        <v>40</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>19</v>
@@ -2111,34 +2145,34 @@
     </row>
     <row r="24" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B24" s="3">
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>19</v>
@@ -2146,22 +2180,22 @@
     </row>
     <row r="25" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B25" s="3">
         <v>3</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>65</v>
+        <v>43</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>15</v>
@@ -2170,10 +2204,10 @@
         <v>16</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>19</v>
@@ -2181,34 +2215,34 @@
     </row>
     <row r="26" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B26" s="3">
         <v>3</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="K26" s="7" t="s">
         <v>19</v>
@@ -2216,34 +2250,34 @@
     </row>
     <row r="27" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B27" s="3">
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>37</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F27" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="K27" s="7" t="s">
         <v>19</v>
@@ -2251,22 +2285,22 @@
     </row>
     <row r="28" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B28" s="3">
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>33</v>
+        <v>43</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>15</v>
@@ -2275,10 +2309,10 @@
         <v>16</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K28" s="7" t="s">
         <v>19</v>
@@ -2286,69 +2320,69 @@
     </row>
     <row r="29" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B29" s="3">
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F29" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="K29" s="11" t="s">
-        <v>117</v>
+        <v>113</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B30" s="3">
         <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>37</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F30" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H30" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="K30" s="7" t="s">
         <v>19</v>
@@ -2356,34 +2390,34 @@
     </row>
     <row r="31" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B31" s="3">
         <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F31" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>122</v>
+        <v>27</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K31" s="7" t="s">
         <v>19</v>
@@ -2391,34 +2425,34 @@
     </row>
     <row r="32" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B32" s="3">
         <v>3</v>
       </c>
       <c r="C32" t="s">
-        <v>37</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>100</v>
+        <v>43</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>84</v>
+      <c r="G32" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>27</v>
+        <v>120</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="K32" s="7" t="s">
         <v>19</v>
@@ -2426,34 +2460,34 @@
     </row>
     <row r="33" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B33" s="3">
         <v>3</v>
       </c>
       <c r="C33" t="s">
-        <v>37</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H33" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="K33" s="7" t="s">
         <v>19</v>
@@ -2461,57 +2495,57 @@
     </row>
     <row r="34" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B34" s="3">
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F34" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H34" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="K34" s="11" t="s">
-        <v>117</v>
+        <v>127</v>
+      </c>
+      <c r="K34" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B35" s="3">
         <v>3</v>
       </c>
       <c r="C35" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>25</v>
+        <v>43</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>33</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>21</v>
@@ -2520,10 +2554,10 @@
         <v>16</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="K35" s="7" t="s">
         <v>19</v>
@@ -2531,22 +2565,22 @@
     </row>
     <row r="36" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B36" s="3">
         <v>3</v>
       </c>
       <c r="C36" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>33</v>
+        <v>43</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>38</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>21</v>
@@ -2555,10 +2589,10 @@
         <v>16</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>136</v>
+        <v>40</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>19</v>
@@ -2566,34 +2600,34 @@
     </row>
     <row r="37" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B37" s="3">
         <v>3</v>
       </c>
       <c r="C37" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H37" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="K37" s="7" t="s">
         <v>19</v>
@@ -2601,104 +2635,104 @@
     </row>
     <row r="38" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B38" s="3">
         <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>37</v>
-      </c>
-      <c r="D38" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F38" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G38" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>16</v>
+        <v>43</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G38" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>139</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>141</v>
+        <v>43</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="K38" s="7" t="s">
-        <v>19</v>
+        <v>43</v>
+      </c>
+      <c r="K38" s="14" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B39" s="3">
         <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>37</v>
-      </c>
-      <c r="D39" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G39" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="H39" s="11" t="s">
-        <v>117</v>
+        <v>43</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K39" s="11" t="s">
-        <v>117</v>
+        <v>142</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B40" s="3">
         <v>3</v>
       </c>
       <c r="C40" t="s">
-        <v>37</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F40" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="K40" s="7" t="s">
         <v>19</v>
@@ -2706,22 +2740,22 @@
     </row>
     <row r="41" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B41" s="3">
         <v>3</v>
       </c>
       <c r="C41" t="s">
-        <v>37</v>
-      </c>
-      <c r="D41" s="11" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E41" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F41" s="20" t="s">
-        <v>87</v>
+      <c r="F41" s="12" t="s">
+        <v>38</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>21</v>
@@ -2730,10 +2764,10 @@
         <v>16</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>149</v>
+        <v>40</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="K41" s="7" t="s">
         <v>19</v>
@@ -2741,101 +2775,101 @@
     </row>
     <row r="42" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B42" s="3">
         <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>37</v>
-      </c>
-      <c r="D42" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F42" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G42" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>16</v>
+        <v>43</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F42" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="G42" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>139</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="K42" s="7" t="s">
-        <v>19</v>
+        <v>43</v>
+      </c>
+      <c r="K42" s="14" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B43" s="3">
         <v>3</v>
       </c>
       <c r="C43" t="s">
-        <v>37</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F43" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="G43" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>117</v>
+        <v>43</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K43" s="11" t="s">
-        <v>117</v>
+        <v>152</v>
+      </c>
+      <c r="K43" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" t="s">
+        <v>43</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E44" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="F44" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="B44" s="3">
-        <v>3</v>
-      </c>
-      <c r="C44" t="s">
-        <v>37</v>
-      </c>
-      <c r="D44" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="J44" s="3" t="s">
         <v>157</v>
@@ -2849,31 +2883,31 @@
         <v>158</v>
       </c>
       <c r="B45" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C45" t="s">
-        <v>37</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E45" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G45" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="F45" s="22" t="s">
+      <c r="J45" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J45" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="K45" s="7" t="s">
         <v>19</v>
@@ -2881,34 +2915,34 @@
     </row>
     <row r="46" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B46" s="3">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>43</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E46" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="B46" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" t="s">
-        <v>37</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E46" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>21</v>
+      <c r="F46" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H46" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K46" s="7" t="s">
         <v>19</v>
@@ -2916,34 +2950,34 @@
     </row>
     <row r="47" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="B47" t="s">
-        <v>37</v>
+        <v>166</v>
+      </c>
+      <c r="B47" s="3">
+        <v>3</v>
       </c>
       <c r="C47" t="s">
-        <v>37</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E47" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F47" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E47" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="F47" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G47" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H47" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>166</v>
+        <v>135</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K47" s="7" t="s">
         <v>19</v>
@@ -2951,34 +2985,34 @@
     </row>
     <row r="48" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B48" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C48" t="s">
-        <v>37</v>
-      </c>
-      <c r="D48" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F48" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H48" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K48" s="7" t="s">
         <v>19</v>
@@ -2986,72 +3020,72 @@
     </row>
     <row r="49" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B49" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C49" t="s">
-        <v>37</v>
-      </c>
-      <c r="D49" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E49" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F49" s="20" t="s">
-        <v>87</v>
+        <v>43</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F49" s="24" t="s">
+        <v>173</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H49" s="19" t="s">
-        <v>172</v>
+      <c r="H49" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>119</v>
+        <v>174</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="K49" s="11" t="s">
-        <v>117</v>
+        <v>175</v>
+      </c>
+      <c r="K49" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C50" t="s">
-        <v>37</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E50" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G50" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>16</v>
+        <v>43</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F50" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G50" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" s="18" t="s">
+        <v>177</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>177</v>
+        <v>112</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K50" s="4" t="s">
         <v>178</v>
+      </c>
+      <c r="K50" s="14" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3059,54 +3093,54 @@
         <v>179</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C51" t="s">
-        <v>37</v>
-      </c>
-      <c r="D51" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F51" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G51" s="18" t="s">
+        <v>181</v>
       </c>
       <c r="H51" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="K51" s="7" t="s">
-        <v>19</v>
+        <v>43</v>
+      </c>
+      <c r="K51" s="4" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B52" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C52" t="s">
-        <v>37</v>
-      </c>
-      <c r="D52" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E52" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F52" s="12" t="s">
         <v>38</v>
-      </c>
-      <c r="F52" s="13" t="s">
-        <v>39</v>
       </c>
       <c r="G52" s="6" t="s">
         <v>15</v>
@@ -3115,10 +3149,10 @@
         <v>16</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="K52" s="7" t="s">
         <v>19</v>
@@ -3126,34 +3160,34 @@
     </row>
     <row r="53" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B53" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C53" t="s">
-        <v>37</v>
-      </c>
-      <c r="D53" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E53" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F53" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G53" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E53" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="F53" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="H53" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="K53" s="7" t="s">
         <v>19</v>
@@ -3161,34 +3195,34 @@
     </row>
     <row r="54" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B54" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C54" t="s">
-        <v>37</v>
-      </c>
-      <c r="D54" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E54" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F54" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G54" s="6" t="s">
-        <v>15</v>
+        <v>43</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F54" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G54" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="H54" s="7" t="s">
         <v>16</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="K54" s="7" t="s">
         <v>19</v>
@@ -3196,34 +3230,34 @@
     </row>
     <row r="55" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="B55" s="3">
-        <v>2.1</v>
-      </c>
-      <c r="C55" s="3">
-        <v>21.1</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F55" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="G55" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H55" s="14" t="s">
-        <v>40</v>
+        <v>194</v>
+      </c>
+      <c r="B55" t="s">
+        <v>43</v>
+      </c>
+      <c r="C55" t="s">
+        <v>43</v>
+      </c>
+      <c r="D55" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F55" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="K55" s="7" t="s">
         <v>19</v>
@@ -3231,34 +3265,34 @@
     </row>
     <row r="56" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B56" s="3">
         <v>2.1</v>
       </c>
       <c r="C56" s="3">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F56" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="G56" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H56" s="14" t="s">
-        <v>40</v>
+      <c r="F56" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H56" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="K56" s="7" t="s">
         <v>19</v>
@@ -3266,7 +3300,7 @@
     </row>
     <row r="57" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B57" s="3">
         <v>2.1</v>
@@ -3275,33 +3309,33 @@
         <v>21</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F57" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="G57" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="H57" s="14" t="s">
-        <v>40</v>
+      <c r="F57" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>169</v>
+        <v>202</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="K57" s="4" t="s">
-        <v>178</v>
+        <v>203</v>
+      </c>
+      <c r="K57" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B58" s="3">
         <v>2.1</v>
@@ -3310,33 +3344,33 @@
         <v>21</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F58" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G58" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H58" s="14" t="s">
-        <v>40</v>
+      <c r="F58" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="G58" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="H58" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="K58" s="7" t="s">
-        <v>19</v>
+        <v>206</v>
+      </c>
+      <c r="K58" s="4" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B59" s="3">
         <v>2.1</v>
@@ -3345,25 +3379,25 @@
         <v>21</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E59" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F59" s="15" t="s">
-        <v>45</v>
+      <c r="F59" s="18" t="s">
+        <v>64</v>
       </c>
       <c r="G59" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H59" s="14" t="s">
-        <v>40</v>
+      <c r="H59" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>204</v>
+        <v>135</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="K59" s="7" t="s">
         <v>19</v>
@@ -3371,7 +3405,7 @@
     </row>
     <row r="60" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B60" s="3">
         <v>2.1</v>
@@ -3380,25 +3414,25 @@
         <v>21</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E60" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F60" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G60" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H60" s="14" t="s">
-        <v>40</v>
+      <c r="F60" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H60" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="K60" s="7" t="s">
         <v>19</v>
@@ -3406,7 +3440,7 @@
     </row>
     <row r="61" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B61" s="3">
         <v>2.1</v>
@@ -3415,25 +3449,25 @@
         <v>21</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F61" s="9" t="s">
-        <v>25</v>
+      <c r="F61" s="17" t="s">
+        <v>60</v>
       </c>
       <c r="G61" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H61" s="14" t="s">
-        <v>40</v>
+      <c r="H61" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>27</v>
+        <v>213</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="K61" s="7" t="s">
         <v>19</v>
@@ -3441,7 +3475,7 @@
     </row>
     <row r="62" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B62" s="3">
         <v>2.1</v>
@@ -3450,25 +3484,25 @@
         <v>21</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E62" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F62" s="19" t="s">
-        <v>69</v>
+      <c r="F62" s="9" t="s">
+        <v>25</v>
       </c>
       <c r="G62" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H62" s="14" t="s">
-        <v>40</v>
+      <c r="H62" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>212</v>
+        <v>27</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="K62" s="7" t="s">
         <v>19</v>
@@ -3476,7 +3510,7 @@
     </row>
     <row r="63" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B63" s="3">
         <v>2.1</v>
@@ -3485,25 +3519,25 @@
         <v>21</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E63" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F63" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="G63" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H63" s="14" t="s">
-        <v>40</v>
+      <c r="F63" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="K63" s="7" t="s">
         <v>19</v>
@@ -3511,7 +3545,7 @@
     </row>
     <row r="64" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B64" s="3">
         <v>2.1</v>
@@ -3520,25 +3554,25 @@
         <v>21</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F64" s="18" t="s">
-        <v>65</v>
+      <c r="F64" s="24" t="s">
+        <v>173</v>
       </c>
       <c r="G64" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H64" s="14" t="s">
-        <v>40</v>
+      <c r="H64" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="K64" s="7" t="s">
         <v>19</v>
@@ -3546,7 +3580,7 @@
     </row>
     <row r="65" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B65" s="3">
         <v>2.1</v>
@@ -3555,25 +3589,25 @@
         <v>21</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E65" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F65" s="18" t="s">
-        <v>65</v>
+      <c r="F65" s="17" t="s">
+        <v>60</v>
       </c>
       <c r="G65" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H65" s="14" t="s">
-        <v>40</v>
+      <c r="H65" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="K65" s="7" t="s">
         <v>19</v>
@@ -3581,7 +3615,7 @@
     </row>
     <row r="66" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B66" s="3">
         <v>2.1</v>
@@ -3590,25 +3624,25 @@
         <v>21</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E66" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F66" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H66" s="14" t="s">
-        <v>40</v>
+      <c r="F66" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H66" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="K66" s="7" t="s">
         <v>19</v>
@@ -3616,34 +3650,34 @@
     </row>
     <row r="67" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B67" s="3">
         <v>2.1</v>
       </c>
       <c r="C67" s="3">
-        <v>21.1</v>
-      </c>
-      <c r="D67" s="16" t="s">
-        <v>49</v>
+        <v>21</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>198</v>
       </c>
       <c r="E67" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F67" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G67" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H67" s="14" t="s">
-        <v>40</v>
+      <c r="F67" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H67" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>109</v>
+        <v>229</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="K67" s="7" t="s">
         <v>19</v>
@@ -3651,7 +3685,7 @@
     </row>
     <row r="68" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B68" s="3">
         <v>2.1</v>
@@ -3659,26 +3693,26 @@
       <c r="C68" s="3">
         <v>21.1</v>
       </c>
-      <c r="D68" s="16" t="s">
-        <v>49</v>
+      <c r="D68" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="E68" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F68" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G68" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H68" s="14" t="s">
-        <v>40</v>
+      <c r="F68" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H68" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>141</v>
+        <v>103</v>
       </c>
       <c r="J68" s="3" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="K68" s="7" t="s">
         <v>19</v>
@@ -3686,7 +3720,7 @@
     </row>
     <row r="69" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B69" s="3">
         <v>2.1</v>
@@ -3694,26 +3728,26 @@
       <c r="C69" s="3">
         <v>21.1</v>
       </c>
-      <c r="D69" s="16" t="s">
-        <v>49</v>
+      <c r="D69" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="E69" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F69" s="19" t="s">
-        <v>69</v>
+      <c r="F69" s="18" t="s">
+        <v>64</v>
       </c>
       <c r="G69" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H69" s="14" t="s">
-        <v>40</v>
+      <c r="H69" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="K69" s="7" t="s">
         <v>19</v>
@@ -3721,7 +3755,7 @@
     </row>
     <row r="70" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B70" s="3">
         <v>2.1</v>
@@ -3729,26 +3763,26 @@
       <c r="C70" s="3">
         <v>21.1</v>
       </c>
-      <c r="D70" s="16" t="s">
-        <v>49</v>
+      <c r="D70" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="E70" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F70" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G70" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H70" s="14" t="s">
-        <v>40</v>
+      <c r="F70" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="J70" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="K70" s="7" t="s">
         <v>19</v>
@@ -3756,7 +3790,7 @@
     </row>
     <row r="71" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B71" s="3">
         <v>2.1</v>
@@ -3764,26 +3798,26 @@
       <c r="C71" s="3">
         <v>21.1</v>
       </c>
-      <c r="D71" s="16" t="s">
-        <v>49</v>
+      <c r="D71" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F71" s="13" t="s">
-        <v>39</v>
+      <c r="F71" s="18" t="s">
+        <v>64</v>
       </c>
       <c r="G71" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H71" s="14" t="s">
-        <v>40</v>
+      <c r="H71" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="K71" s="7" t="s">
         <v>19</v>
@@ -3791,7 +3825,7 @@
     </row>
     <row r="72" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B72" s="3">
         <v>2.1</v>
@@ -3799,26 +3833,26 @@
       <c r="C72" s="3">
         <v>21.1</v>
       </c>
-      <c r="D72" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F72" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="G72" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H72" s="14" t="s">
+      <c r="D72" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G72" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H72" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="I72" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I72" s="3" t="s">
-        <v>141</v>
-      </c>
       <c r="J72" s="3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="K72" s="7" t="s">
         <v>19</v>
@@ -3826,7 +3860,7 @@
     </row>
     <row r="73" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B73" s="3">
         <v>2.1</v>
@@ -3834,26 +3868,26 @@
       <c r="C73" s="3">
         <v>21.1</v>
       </c>
-      <c r="D73" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="E73" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F73" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="G73" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H73" s="14" t="s">
-        <v>40</v>
+      <c r="D73" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F73" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G73" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H73" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>238</v>
+        <v>135</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="K73" s="7" t="s">
         <v>19</v>
@@ -3861,7 +3895,7 @@
     </row>
     <row r="74" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B74" s="3">
         <v>2.1</v>
@@ -3869,32 +3903,67 @@
       <c r="C74" s="3">
         <v>21.1</v>
       </c>
-      <c r="D74" s="16" t="s">
-        <v>49</v>
+      <c r="D74" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F74" s="19" t="s">
-        <v>69</v>
+      <c r="F74" s="21" t="s">
+        <v>155</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H74" s="14" t="s">
-        <v>40</v>
+      <c r="H74" s="13" t="s">
+        <v>39</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J74" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="K74" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B75" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="C75" s="3">
+        <v>21.1</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F75" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G75" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H75" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="K75" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
add dmri known issue
</commit_message>
<xml_diff>
--- a/tools/latest.xlsx
+++ b/tools/latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10911"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E26D21-8B95-B14D-B802-7E1B2D4E0996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD37F8C5-7917-F24A-99BC-E4134BFF0826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="237">
   <si>
     <t>Name</t>
   </si>
@@ -717,13 +717,22 @@
   </si>
   <si>
     <t>A future release will include reliability codes integrated into the primary coding dataset. Until then, users must perform this integration manually: see the ERICA Data Warning for instructions. Instructions include cleaning the current files to exclude n=44 participants with incorrect code values (data entry/form errors), capping `b_raw` values at 3.0 (n=3 participants), and removing the “Locomotor Ability” field (`mh_cg_erica_3_9m_locomotor_ability`), which has errors, also to be corrected in the next release.</t>
+  </si>
+  <si>
+    <t>[DATA ISSUE] Diffusion MRI</t>
+  </si>
+  <si>
+    <t>dMRI metadata</t>
+  </si>
+  <si>
+    <t>`LargeDelta` and `SmallDelta` in the sidecars currently are set to vendor-specific values (which aren't always correct because the models have their own values) and ﻿will be updated to reflect accurate values.﻿ ﻿</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -740,6 +749,13 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="21">
@@ -857,7 +873,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -922,6 +938,7 @@
     <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1261,7 +1278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:M70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.33203125" customWidth="1"/>
@@ -3709,7 +3726,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="65" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:13" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>220</v>
       </c>
@@ -3747,7 +3764,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="66" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:13" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>221</v>
       </c>
@@ -3785,7 +3802,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="67" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>222</v>
       </c>
@@ -3823,7 +3840,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:13" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>227</v>
       </c>
@@ -3861,7 +3878,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:13" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>230</v>
       </c>
@@ -3899,7 +3916,36 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="70" spans="1:13" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>234</v>
+      </c>
+      <c r="E70" s="22"/>
+      <c r="F70" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G70" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="H70" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I70" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="J70" t="s">
+        <v>235</v>
+      </c>
+      <c r="K70" t="s">
+        <v>236</v>
+      </c>
+      <c r="L70" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="M70" s="22" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>